<commit_message>
docs(media): add tracker handover sheet
</commit_message>
<xml_diff>
--- a/docs/superpowers/plans/2026-09-08-model-agnostic-atomic-media-platform-tracker.xlsx
+++ b/docs/superpowers/plans/2026-09-08-model-agnostic-atomic-media-platform-tracker.xlsx
@@ -7,14 +7,15 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tasks" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Steps" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Handover" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tasks" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Steps" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tasks'!$A$2:$K$20</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Steps'!$A$1:$I$129</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Tasks'!$A$2:$K$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Steps'!$A$1:$I$129</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -25,7 +26,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -66,8 +67,34 @@
       <color rgb="FF808080"/>
       <sz val="9"/>
     </font>
+    <font>
+      <b val="1"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <b val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color theme="1"/>
+      <sz val="10"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -99,8 +126,23 @@
         <fgColor rgb="FFFCE5CD"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E78"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9EAF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -123,11 +165,16 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <bottom style="thin">
+        <color rgb="00D9E2F3"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -165,6 +212,18 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -923,6 +982,194 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:B16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="115" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="18" t="inlineStr">
+        <is>
+          <t>Atomic Media handover</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="19" t="inlineStr">
+        <is>
+          <t>Created for the next agent. Continue from the tracker, not from memory.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="20" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B4" s="20" t="inlineStr">
+        <is>
+          <t>Current value</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="34" customHeight="1">
+      <c r="A5" s="21" t="inlineStr">
+        <is>
+          <t>Repository</t>
+        </is>
+      </c>
+      <c r="B5" s="22" t="inlineStr">
+        <is>
+          <t>C:\Users\Warwick\.codex\.chatgpt-projects\g-p-6a89e2d97fa08191bee04f4c7a2099a9\Atomic-Chat</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="34" customHeight="1">
+      <c r="A6" s="21" t="inlineStr">
+        <is>
+          <t>Branch</t>
+        </is>
+      </c>
+      <c r="B6" s="22" t="inlineStr">
+        <is>
+          <t>feature/atomic-code-foundation</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="34" customHeight="1">
+      <c r="A7" s="21" t="inlineStr">
+        <is>
+          <t>Latest local commit</t>
+        </is>
+      </c>
+      <c r="B7" s="22" t="inlineStr">
+        <is>
+          <t>166b5758f chore(guard): re-baseline Atomic Media protected hashes</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="34" customHeight="1">
+      <c r="A8" s="21" t="inlineStr">
+        <is>
+          <t>Where to start</t>
+        </is>
+      </c>
+      <c r="B8" s="22" t="inlineStr">
+        <is>
+          <t>Task 0 remains In progress. make verify is the active gate before Task 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="34" customHeight="1">
+      <c r="A9" s="21" t="inlineStr">
+        <is>
+          <t>Tracker progress noted</t>
+        </is>
+      </c>
+      <c r="B9" s="22" t="inlineStr">
+        <is>
+          <t>Q1 is Answered. T00-S01 through T00-S07 are Done. Task 0 is In progress.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="34" customHeight="1">
+      <c r="A10" s="21" t="inlineStr">
+        <is>
+          <t>Do not commit</t>
+        </is>
+      </c>
+      <c r="B10" s="23" t="inlineStr">
+        <is>
+          <t>downloads/index.html; extensions/yarn.lock; src-tauri/icons/icon.png; web-app/src/lib/models.ts; web-app/src/hooks/useModelSources.ts; web-app/src/lib/__tests__/models.test.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="34" customHeight="1">
+      <c r="A11" s="21" t="inlineStr">
+        <is>
+          <t>Verification passed</t>
+        </is>
+      </c>
+      <c r="B11" s="22" t="inlineStr">
+        <is>
+          <t>make test-selective-v2032 exits 0; node guard tests pass 4/4; node scripts/verify-selective-v2032.mjs prints boundaries verified.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="34" customHeight="1">
+      <c r="A12" s="21" t="inlineStr">
+        <is>
+          <t>Verification blocker</t>
+        </is>
+      </c>
+      <c r="B12" s="23" t="inlineStr">
+        <is>
+          <t>make verify reaches test-quality and fails on pre-existing call-only assertion findings. Fix or allowlist that guard before Task 0 can be marked Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="34" customHeight="1">
+      <c r="A13" s="21" t="inlineStr">
+        <is>
+          <t>Local tool setup</t>
+        </is>
+      </c>
+      <c r="B13" s="22" t="inlineStr">
+        <is>
+          <t>GNU Make is installed at C:\Users\Warwick\AppData\Local\Programs\GnuWin32\bin\make.exe. yarn.cmd shim there delegates to Corepack Yarn 4.5.3.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="34" customHeight="1">
+      <c r="A14" s="21" t="inlineStr">
+        <is>
+          <t>Command note</t>
+        </is>
+      </c>
+      <c r="B14" s="22" t="inlineStr">
+        <is>
+          <t>In this Codex shell, prepend PATH with C:\Users\Warwick\AppData\Local\Programs\GnuWin32\bin before running make. New terminals should inherit the user PATH.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="34" customHeight="1">
+      <c r="A15" s="21" t="inlineStr">
+        <is>
+          <t>Last make verify output</t>
+        </is>
+      </c>
+      <c r="B15" s="22" t="inlineStr">
+        <is>
+          <t>Lint produced 13 warnings, typecheck completed, then test-quality failed with call-only-assertions in nine existing test files.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="34" customHeight="1">
+      <c r="A16" s="21" t="inlineStr">
+        <is>
+          <t>Next action</t>
+        </is>
+      </c>
+      <c r="B16" s="23" t="inlineStr">
+        <is>
+          <t>Resolve the test-quality guard failures, rerun make verify, then update Task 0 status only if the full gate is green.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:K20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
@@ -1828,7 +2075,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6622,7 +6869,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6869,7 +7116,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
docs(media): refresh tracker handover
</commit_message>
<xml_diff>
--- a/docs/superpowers/plans/2026-09-08-model-agnostic-atomic-media-platform-tracker.xlsx
+++ b/docs/superpowers/plans/2026-09-08-model-agnostic-atomic-media-platform-tracker.xlsx
@@ -174,7 +174,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -223,6 +223,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1003,6 +1006,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="20" t="inlineStr">
         <is>
@@ -1047,7 +1051,7 @@
       </c>
       <c r="B7" s="22" t="inlineStr">
         <is>
-          <t>166b5758f chore(guard): re-baseline Atomic Media protected hashes</t>
+          <t>f4f27751a test: document existing quality guard exceptions</t>
         </is>
       </c>
     </row>
@@ -1059,7 +1063,7 @@
       </c>
       <c r="B8" s="22" t="inlineStr">
         <is>
-          <t>Task 0 remains In progress. make verify is the active gate before Task 1.</t>
+          <t>Task 0 remains In progress. make verify is still the active gate before Task 1.</t>
         </is>
       </c>
     </row>
@@ -1095,7 +1099,7 @@
       </c>
       <c r="B11" s="22" t="inlineStr">
         <is>
-          <t>make test-selective-v2032 exits 0; node guard tests pass 4/4; node scripts/verify-selective-v2032.mjs prints boundaries verified.</t>
+          <t>make test-quality now exits 0 after documenting seven existing call-only assertion exceptions. make test-selective-v2032 exits 0; node guard tests pass 4/4; node scripts/verify-selective-v2032.mjs prints boundaries verified.</t>
         </is>
       </c>
     </row>
@@ -1107,7 +1111,7 @@
       </c>
       <c r="B12" s="23" t="inlineStr">
         <is>
-          <t>make verify reaches test-quality and fails on pre-existing call-only assertion findings. Fix or allowlist that guard before Task 0 can be marked Done.</t>
+          <t>make verify now reaches test-coverage-critical and fails with 4 tests: main.test.tsx timeout; formatDate old-date timezone expectation; two huggingface-conversion assertions in the model-catalog/GGUF area that is already dirty and forbidden to commit in this task.</t>
         </is>
       </c>
     </row>
@@ -1143,7 +1147,7 @@
       </c>
       <c r="B15" s="22" t="inlineStr">
         <is>
-          <t>Lint produced 13 warnings, typecheck completed, then test-quality failed with call-only-assertions in nine existing test files.</t>
+          <t>Lint produced 13 warnings, typecheck passed, test-quality passed, hardening contracts passed, then coverage failed: 3 files failed, 4 tests failed, 2227 passed, 16 skipped.</t>
         </is>
       </c>
     </row>
@@ -1155,7 +1159,7 @@
       </c>
       <c r="B16" s="23" t="inlineStr">
         <is>
-          <t>Resolve the test-quality guard failures, rerun make verify, then update Task 0 status only if the full gate is green.</t>
+          <t>Do not start Task 1 until make verify is green. Resolve or coordinate the existing coverage failures without committing the six forbidden dirty paths unless the user changes that rule.</t>
         </is>
       </c>
     </row>
@@ -7122,7 +7126,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -7474,6 +7478,28 @@
       <c r="F13" s="15" t="n"/>
       <c r="G13" s="15" t="n"/>
     </row>
+    <row r="14">
+      <c r="A14" s="24" t="inlineStr">
+        <is>
+          <t>make verify after f4f27751a</t>
+        </is>
+      </c>
+      <c r="B14" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C14" s="24" t="inlineStr">
+        <is>
+          <t>FAIL at test-coverage-critical: main.test.tsx timeout; formatDate timezone expectation; two huggingface-conversion failures in current model-catalog dirty area.</t>
+        </is>
+      </c>
+      <c r="D14" s="24" t="inlineStr">
+        <is>
+          <t>Task 0 remains In progress; Task 1 blocked.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="E2:E13" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">

</xml_diff>

<commit_message>
fix(verify): make `make verify` pass on Windows for Task 0
The Rust desktop tests had never run on Windows before (linking was
blocked), so two Windows-only test issues surfaced once linking worked:

- utils path.rs: the "a path with nothing existing is returned unchanged"
  test assumed Unix semantics — on Windows a leading `/` canonicalizes to
  the current drive root, so the tail is re-attached. Gate that assertion
  to cfg(unix) like its two sibling tests, and add a cfg(windows)
  equivalent that reaches the same state via an unmounted drive letter.
- web-app vitest.config.ts: under the coverage run, one instrumented
  worker per core starves otherwise sub-second tests past the 5s default,
  so they time out under load. Raise testTimeout to 30s (vitest's own
  recommended remedy) so a slow-to-schedule test is not read as a hang.

Also mark Task 0 Done in the Atomic Media tracker: full `make verify`
now exits 0.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/superpowers/plans/2026-09-08-model-agnostic-atomic-media-platform-tracker.xlsx
+++ b/docs/superpowers/plans/2026-09-08-model-agnostic-atomic-media-platform-tracker.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Handover" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tasks" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Steps" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Handover" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Tasks" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Steps" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Decisions" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Evidence" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Tasks'!$A$2:$K$20</definedName>
@@ -1006,7 +1006,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="20" t="inlineStr">
         <is>
@@ -1063,7 +1062,7 @@
       </c>
       <c r="B8" s="22" t="inlineStr">
         <is>
-          <t>Task 0 remains In progress. make verify is still the active gate before Task 1.</t>
+          <t>Task 0 gate met: make verify exits 0 in the working tree (2026-09-09). Next work is Task 1 (T01-S01) once the enabling changes are committed. Do not start Task 1 until Task 0 changes are committed.</t>
         </is>
       </c>
     </row>
@@ -1075,7 +1074,7 @@
       </c>
       <c r="B9" s="22" t="inlineStr">
         <is>
-          <t>Q1 is Answered. T00-S01 through T00-S07 are Done. Task 0 is In progress.</t>
+          <t>Q1 Answered. T00-S01..S07 Done. Task 0 marked Done 2026-09-09 on green make verify (working tree; uncommitted).</t>
         </is>
       </c>
     </row>
@@ -1111,7 +1110,7 @@
       </c>
       <c r="B12" s="23" t="inlineStr">
         <is>
-          <t>make verify now reaches test-coverage-critical and fails with 4 tests: main.test.tsx timeout; formatDate old-date timezone expectation; two huggingface-conversion assertions in the model-catalog/GGUF area that is already dirty and forbidden to commit in this task.</t>
+          <t>RESOLVED 2026-09-09. Prior blocker was Rust desktop test linking (LNK1104 ucrt.lib) plus, once linking worked, two Windows-only test issues (shell contract needed printf on PATH; utils path.rs test assumed Unix / semantics) and web-coverage worker-starvation timeouts. All fixed. See Tasks!K3.</t>
         </is>
       </c>
     </row>
@@ -1147,7 +1146,7 @@
       </c>
       <c r="B15" s="22" t="inlineStr">
         <is>
-          <t>Lint produced 13 warnings, typecheck passed, test-quality passed, hardening contracts passed, then coverage failed: 3 files failed, 4 tests failed, 2227 passed, 16 skipped.</t>
+          <t>2026-09-09 make verify EXITCODE=0. Environment: run from a VS x64 developer shell (vcvars64.bat) with a printf.exe-only directory appended to PATH (Git usr/bin as a whole must NOT be added, or make switches to sh and breaks the PowerShell stub-resources recipe, and Git link.exe shadows MSVC link.exe).</t>
         </is>
       </c>
     </row>
@@ -1277,7 +1276,7 @@
       </c>
       <c r="E3" s="13" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F3" s="13" t="n"/>
@@ -1299,7 +1298,7 @@
       </c>
       <c r="K3" s="15" t="inlineStr">
         <is>
-          <t>Q1 answered 2026-09-08: Option A (re-baseline). Gate is open; proceed at T00-S02.</t>
+          <t>Q1 answered 2026-09-08: Option A (re-baseline). Gate is open; proceed at T00-S02. | 2026-09-09: make verify exits 0 (full green). Web coverage 2234 passed/16 skipped; extension 250+276; Rust 487+12+167+205+28+4; coverage floor 9 files; selective v2.0.32 boundaries verified. GREEN DEPENDS ON uncommitted working-tree fixes (previous agent test fixes + this session: src-tauri/utils/src/path.rs Windows test gating, web-app/vitest.config.ts testTimeout 30s) AND a VS x64 dev env (vcvars64.bat) plus a printf.exe-only dir on PATH so link.exe finds ucrt.lib and make stays on cmd for stub-resources. Nothing committed pending user authorization.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(tracker): mark Task 1 Done with its commit SHA
Records c62b11da8 against T01-S06 and Task 1, and carries the handover
forward to T02-S01.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/superpowers/plans/2026-09-08-model-agnostic-atomic-media-platform-tracker.xlsx
+++ b/docs/superpowers/plans/2026-09-08-model-agnostic-atomic-media-platform-tracker.xlsx
@@ -1050,7 +1050,7 @@
       </c>
       <c r="B7" s="22" t="inlineStr">
         <is>
-          <t>8ec82bef3 merge: integrate remote task0 quality-gate exceptions (pushed to origin)</t>
+          <t>c62b11da8 feat(media): add model-agnostic media contract v2 (local, not yet pushed)</t>
         </is>
       </c>
     </row>
@@ -1062,7 +1062,7 @@
       </c>
       <c r="B8" s="22" t="inlineStr">
         <is>
-          <t>Task 0 Done and committed (9e8249046, pushed in 8ec82bef3). Task 1 code complete through T01-S05 in the working tree and uncommitted; next action is T01-S06 (commit) once the user authorises it, then Task 2 (T02-S01).</t>
+          <t>Task 0 Done and pushed (9e8249046 in merge 8ec82bef3). Task 1 Done and committed locally (c62b11da8); not yet pushed. Next work is Task 2, starting at T02-S01: capture a v1 capabilities payload as a fixture. Live worker capture is preferred; the laptop fallback is MediaStudio.test.tsx:9-58 - record which source was used.</t>
         </is>
       </c>
     </row>
@@ -1074,7 +1074,7 @@
       </c>
       <c r="B9" s="22" t="inlineStr">
         <is>
-          <t>Q1 Answered. T00-S01..S07 Done. Task 0 Done. T01-S01..S05 Done 2026-09-09. T01-S06 (commit) outstanding.</t>
+          <t>Q1 Answered. T00-S01..S07 Done, Task 0 Done. T01-S01..S06 Done, Task 1 Done 2026-09-09 on green make verify, committed c62b11da8. Next not-done step is T02-S01.</t>
         </is>
       </c>
     </row>
@@ -1158,7 +1158,7 @@
       </c>
       <c r="B16" s="23" t="inlineStr">
         <is>
-          <t>Commit the Task 1 contract when the user authorises it (feat(media): add model-agnostic media contract v2), staging ONLY web-app/src/services/media/contract/** and the tracker. Then Task 2 (T02-S01): capture a v1 capabilities payload as a fixture. Resolve the plan's modulus tie-break contradiction with the user before Task 2's parity test is written.</t>
+          <t>Start Task 2 at T02-S01. Before T02-S02 writes the parity test, settle the plan's self-contradictory modulus tie-break text with the user ("19 -&gt; 21" vs "ties round down"): the contract implements round-down, matching v1 nearestFrame. Also decide whether to push feature/atomic-code-foundation - c62b11da8 is local only.</t>
         </is>
       </c>
     </row>
@@ -1325,7 +1325,7 @@
       </c>
       <c r="E4" s="13" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F4" s="13" t="n"/>
@@ -1339,7 +1339,11 @@
           <t>Upcaster round-trip tests green</t>
         </is>
       </c>
-      <c r="I4" s="13" t="n"/>
+      <c r="I4" s="13" t="inlineStr">
+        <is>
+          <t>c62b11da8</t>
+        </is>
+      </c>
       <c r="J4" s="14" t="inlineStr">
         <is>
           <t>Pure types + validateParams. No UI change, no I/O.</t>
@@ -1347,7 +1351,7 @@
       </c>
       <c r="K4" s="15" t="inlineStr">
         <is>
-          <t>2026-09-09: T01-S01..S05 Done. Contract lives in web-app/src/services/media/contract/ (tasks.ts, params.ts, models.ts, jobs.ts, index.ts + __tests__/params.test.ts). 45 focused tests pass; full make verify EXIT 0. Only T01-S06 (commit) outstanding, which needs user authorisation. Open question for the user: the plan Step 1 text contradicts itself on modulus tie-breaking ("19 -&gt; 21" vs "ties round down"); implemented round-down to match v1 nearestFrame and keep the Task 2 parity test valid.</t>
+          <t>2026-09-09: Task 1 complete, T01-S01..S06 all Done. Contract in web-app/src/services/media/contract/ (tasks.ts, params.ts, models.ts, jobs.ts, index.ts + __tests__/params.test.ts). 45 focused tests pass; full make verify EXIT 0. Committed c62b11da8 (local; not yet pushed). OPEN QUESTION for the user: the plan Step 1 text contradicts itself on modulus tie-breaking ("19 -&gt; 21" vs "ties round down"); round-down was implemented to match v1 nearestFrame and keep the Task 2 parity test valid. Settle this before T02-S02 writes that parity test.</t>
         </is>
       </c>
     </row>
@@ -2638,7 +2642,7 @@
       </c>
       <c r="E14" s="13" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F14" s="13" t="n"/>
@@ -2654,7 +2658,7 @@
       </c>
       <c r="I14" s="15" t="inlineStr">
         <is>
-          <t>Awaiting user authorisation. Do not stage the pre-existing dirty paths.</t>
+          <t>2026-09-09: committed c62b11da8 "feat(media): add model-agnostic media contract v2". 7 files, 1292 insertions - the six contract files plus this tracker. The 11 pre-existing dirty paths were left unstaged and are still dirty.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(tracker): add the working agreement and refresh stale README guidance
The user has no coding experience, so the tracker cannot assume he will know
when a commit, push or decision is due. Adds a WORKING AGREEMENT block to the
Handover sheet making the obligation explicit and one-directional: the agent
may not commit, push, re-baseline the guard or change scope without specific
authorisation, AND the agent must proactively say when an action is due rather
than waiting to be asked. Includes the per-step process, concrete wording for
asking, and the current eleven never-stage paths.

Also corrects two README lines that would now misdirect a fresh agent: it
still declared `make verify` RED because of a13b71a83 (Task 0 closed that,
though a clean clone remains red pending Q6), and it listed a four-path dirty
set that no longer matches the tree.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/superpowers/plans/2026-09-08-model-agnostic-atomic-media-platform-tracker.xlsx
+++ b/docs/superpowers/plans/2026-09-08-model-agnostic-atomic-media-platform-tracker.xlsx
@@ -593,7 +593,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G38"/>
+  <dimension ref="A1:G42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -683,7 +683,7 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Task 0 is a hard gate. `make verify` is currently RED because commit a13b71a83 changed 8 of the 11 files frozen in scripts/selective-v2032-protected.json. Nothing downstream can be verified until Task 0 lands.</t>
+          <t>Task 0 is a hard gate and it is now CLOSED. It was red because commit a13b71a83 changed 8 of the 11 files frozen in scripts/selective-v2032-protected.json; they were re-baselined and `make verify` exits 0 (2026-09-09). Caveat: green depends on uncommitted model-catalog/GGUF test fixes still sitting in the working tree, so a FRESH CLONE is still red. See Decision Q6.</t>
         </is>
       </c>
     </row>
@@ -695,7 +695,7 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Decision Q1 on the Decisions sheet blocks Task 0. It is the user's call, not yours. Do not guess it.</t>
+          <t>Decision Q1 is answered (Option A, 2026-09-08). Q2-Q6 on the Decisions sheet are still OPEN and are the user's call, not yours. Do not guess one. They only bite when their own task comes up.</t>
         </is>
       </c>
     </row>
@@ -731,7 +731,7 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Never commit the four pre-existing dirty paths: downloads/index.html, extensions/yarn.lock, src-tauri/icons/icon.png, web-app/src/containers/DownloadManegement.tsx.</t>
+          <t>Never commit the pre-existing dirty paths. As of 2026-09-09 there are eleven: downloads/index.html, extensions/yarn.lock, src-tauri/Cargo.lock, src-tauri/icons/icon.png, web-app/src/hooks/useModelSources.ts, web-app/src/lib/models.ts, web-app/src/lib/__tests__/models.test.ts, web-app/src/routes/hub/__tests__/huggingface-conversion.test.ts, web-app/src/services/models/default.ts, web-app/src/utils/__tests__/formatDate.test.ts, web-app/src/utils/getModelToStart.test.ts.</t>
         </is>
       </c>
     </row>
@@ -972,6 +972,37 @@
       <c r="B38" s="7">
         <f>COUNTIF(Decisions!F2:F7,"Open")</f>
         <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>AGENTS: WORKING AGREEMENT (see the Handover sheet for the full version)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>7.</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>You may NOT commit, push, re-baseline the protected guard, or change scope without the user authorising that specific action. Approval for one action is never approval for the next.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>8.</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>The user has NO coding experience. Do not wait to be told when to commit, push, or decide - he will not know, and his silence is not an instruction to wait. YOU must raise it, in plain language, every time the normal process says an action is due. See the WORKING AGREEMENT block on the Handover sheet.</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -985,7 +1016,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1159,6 +1190,102 @@
       <c r="B16" s="23" t="inlineStr">
         <is>
           <t>Start Task 2 at T02-S01. Before T02-S02 writes the parity test, settle the plan's self-contradictory modulus tie-break text with the user ("19 -&gt; 21" vs "ties round down"): the contract implements round-down, matching v1 nearestFrame. Also decide whether to push feature/atomic-code-foundation - c62b11da8 is local only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="20" t="inlineStr">
+        <is>
+          <t>WORKING AGREEMENT</t>
+        </is>
+      </c>
+      <c r="B18" s="20" t="inlineStr">
+        <is>
+          <t>How to work with Warwick. This is not optional and it does not expire.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="21" t="inlineStr">
+        <is>
+          <t>Who authorises what</t>
+        </is>
+      </c>
+      <c r="B19" s="22" t="inlineStr">
+        <is>
+          <t>The agent must NEVER commit, push, force-push, re-baseline the protected-surface guard, switch or create branches, or change the scope of a task without the user authorising that specific action first. Approval for one action is not approval for the next one.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="21" t="inlineStr">
+        <is>
+          <t>The user is not a coder</t>
+        </is>
+      </c>
+      <c r="B20" s="22" t="inlineStr">
+        <is>
+          <t>Warwick has no coding experience. He should NOT be expected to know when a commit, a push, or a decision is due, and his silence is not an instruction to wait. The obligation to raise it sits with the AGENT, every time. Never leave finished, verified work sitting there because nobody asked for it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="21" t="inlineStr">
+        <is>
+          <t>So the agent must prompt</t>
+        </is>
+      </c>
+      <c r="B21" s="22" t="inlineStr">
+        <is>
+          <t>At every point where the normal process says an action is due, say so in plain language, unprompted: what stage we are at, what the normal next step is, and what you need from him (usually a yes, or an answer to an open decision). If he has not asked for something that clearly should have happened by now - a commit after a green make verify, a push after a task is committed, an answer to a decision that is now blocking - remind him and say why it matters.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="21" t="inlineStr">
+        <is>
+          <t>The normal process, per step</t>
+        </is>
+      </c>
+      <c r="B22" s="22" t="inlineStr">
+        <is>
+          <t>Write a failing test -&gt; run it and confirm it fails for the RIGHT reason -&gt; implement -&gt; focused tests green -&gt; full make verify green -&gt; THEN ask the user to authorise the commit -&gt; update this tracker -&gt; ask whether to push. A step is Done only when its stated command has actually been run and passed. Never mark Done on partial success; record which phase failed instead.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="21" t="inlineStr">
+        <is>
+          <t>How to ask, concretely</t>
+        </is>
+      </c>
+      <c r="B23" s="22" t="inlineStr">
+        <is>
+          <t>Example wording after a green verify: "This is the point where we would normally commit. The change is X, the verification is Y, and I would stage only these files with this commit message. Do you want me to commit it? After that the usual next step is pushing to origin - tell me if you want that too." Name the files and the message so he can approve without reading any code. Explain trade-offs in plain terms, not in jargon.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="21" t="inlineStr">
+        <is>
+          <t>Open decisions are his call</t>
+        </is>
+      </c>
+      <c r="B24" s="22" t="inlineStr">
+        <is>
+          <t>Q2-Q6 on the Decisions sheet belong to the user. NEVER guess one. When work reaches a point where an open decision blocks it, stop, ask, and explain in plain language what each option would mean for him and what it would cost to change later. Also flag any contradiction found in the plan itself rather than quietly picking a side - say which side you picked and why.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="21" t="inlineStr">
+        <is>
+          <t>Never stage these paths</t>
+        </is>
+      </c>
+      <c r="B25" s="22" t="inlineStr">
+        <is>
+          <t>These are pre-existing dirty files that belong to other in-flight work (Decision Q6). Leave them dirty and unstaged unless the user specifically authorises otherwise: downloads/index.html; extensions/yarn.lock; src-tauri/Cargo.lock; src-tauri/icons/icon.png; web-app/src/hooks/useModelSources.ts; web-app/src/lib/models.ts; web-app/src/lib/__tests__/models.test.ts; web-app/src/routes/hub/__tests__/huggingface-conversion.test.ts; web-app/src/services/models/default.ts; web-app/src/utils/__tests__/formatDate.test.ts; web-app/src/utils/getModelToStart.test.ts</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(tracker): mark Task 2 Done and correct the clean-checkout record
Records Task 2 complete with its commit SHAs, fills in Evidence rows 1, 2, 3 and
5 from the runs that actually happened, and voids row 6 whose premise no longer
holds now that the pre-existing dirty paths have been resolved.

Adds Decision D2 as an explicit correction. The tracker attributed the red
clean-checkout solely to the uncommitted model-catalog/GGUF fixes under Q6.
There were two independent causes, and committing those files was necessary but
not sufficient - the missing generated app icons would have failed a fresh clone
regardless. Left as written, the next agent would have believed one fix covered
it. A clean clone is now proven green from scratch rather than inferred.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/superpowers/plans/2026-09-08-model-agnostic-atomic-media-platform-tracker.xlsx
+++ b/docs/superpowers/plans/2026-09-08-model-agnostic-atomic-media-platform-tracker.xlsx
@@ -1081,7 +1081,7 @@
       </c>
       <c r="B7" s="22" t="inlineStr">
         <is>
-          <t>c62b11da8 feat(media): add model-agnostic media contract v2 (local, not yet pushed)</t>
+          <t>c54856d2e fix(verify): stop icon generation from degrading the icon.png master</t>
         </is>
       </c>
     </row>
@@ -1093,7 +1093,7 @@
       </c>
       <c r="B8" s="22" t="inlineStr">
         <is>
-          <t>Task 0 Done and pushed (9e8249046 in merge 8ec82bef3). Task 1 Done and committed locally (c62b11da8); not yet pushed. Next work is Task 2, starting at T02-S01: capture a v1 capabilities payload as a fixture. Live worker capture is preferred; the laptop fallback is MediaStudio.test.tsx:9-58 - record which source was used.</t>
+          <t>Tasks 0, 1 and 2 are all Done and committed. Next work is Task 3 (T03-S01): write the shared adapter conformance suite FIRST, parameterised over an adapter factory plus a mock transport - every later adapter must pass it unmodified.</t>
         </is>
       </c>
     </row>
@@ -1105,7 +1105,7 @@
       </c>
       <c r="B9" s="22" t="inlineStr">
         <is>
-          <t>Q1 Answered. T00-S01..S07 Done, Task 0 Done. T01-S01..S06 Done, Task 1 Done 2026-09-09 on green make verify, committed c62b11da8. Next not-done step is T02-S01.</t>
+          <t>Q1 Answered. Task 0 Done. Task 1 Done (c62b11da8). Task 2 Done (8ca22ff6e + isolated re-baseline 59ee8b7fb). D1 and D2 recorded on the Decisions sheet. Q2-Q6 still Open. Next not-done step: T03-S01.</t>
         </is>
       </c>
     </row>
@@ -1129,7 +1129,7 @@
       </c>
       <c r="B11" s="22" t="inlineStr">
         <is>
-          <t>make test-quality now exits 0 after documenting seven existing call-only assertion exceptions. make test-selective-v2032 exits 0; node guard tests pass 4/4; node scripts/verify-selective-v2032.mjs prints boundaries verified.</t>
+          <t>make verify exit 0 on the working tree and, as of 2026-09-09, on a FROM-SCRATCH CLEAN CLONE - the clean-checkout gap is closed and proven, not inferred. See Evidence rows 2 and 5 and Decision D2.</t>
         </is>
       </c>
     </row>
@@ -1141,7 +1141,7 @@
       </c>
       <c r="B12" s="23" t="inlineStr">
         <is>
-          <t>RESOLVED 2026-09-09. Prior blocker was Rust desktop test linking (LNK1104 ucrt.lib) plus, once linking worked, two Windows-only test issues (shell contract needed printf on PATH; utils path.rs test assumed Unix / semantics) and web-coverage worker-starvation timeouts. All fixed. See Tasks!K3.</t>
+          <t>None. The two historic blockers are both fixed: the uncommitted model-catalog/GGUF test fixes are committed, and the missing generated app icons are now produced by the make app-icons target.</t>
         </is>
       </c>
     </row>
@@ -1189,7 +1189,7 @@
       </c>
       <c r="B16" s="23" t="inlineStr">
         <is>
-          <t>Start Task 2 at T02-S01. Before T02-S02 writes the parity test, settle the plan's self-contradictory modulus tie-break text with the user ("19 -&gt; 21" vs "ties round down"): the contract implements round-down, matching v1 nearestFrame. Also decide whether to push feature/atomic-code-foundation - c62b11da8 is local only.</t>
+          <t>Start Task 3 at T03-S01. Note the conformance suite is the deliverable that constrains every future provider, so write it before the adapter. Q2-Q6 remain the user's call and are not needed for Task 3.</t>
         </is>
       </c>
     </row>
@@ -1505,7 +1505,7 @@
       </c>
       <c r="E5" s="13" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F5" s="13" t="n"/>
@@ -1519,7 +1519,11 @@
           <t>Upcaster round-trip tests green</t>
         </is>
       </c>
-      <c r="I5" s="13" t="n"/>
+      <c r="I5" s="13" t="inlineStr">
+        <is>
+          <t>8ca22ff6e (+ 59ee8b7fb guard re-baseline)</t>
+        </is>
+      </c>
       <c r="J5" s="14" t="inlineStr">
         <is>
           <t>Live worker capture preferred for the fixture; the fixture at MediaStudio.test.tsx:9-58 is the laptop fallback. Deletes ATOMIC_MEDIA_DEFAULT_VIDEO_REQUEST.</t>
@@ -3101,7 +3105,7 @@
       </c>
       <c r="E22" s="13" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F22" s="13" t="n"/>
@@ -3117,7 +3121,7 @@
       </c>
       <c r="I22" s="15" t="inlineStr">
         <is>
-          <t>Awaiting T02-S06 and user authorisation to commit.</t>
+          <t>2026-09-09: committed 8ca22ff6e "feat(media): upcast v1 worker capabilities to contract v2" (contract work + the C8 removal + fixture), then 59ee8b7fb as the isolated guard re-baseline per Q1. make verify exit 0; web coverage 2319 passed/16 skipped, up from 2279 by the 40 tests added.</t>
         </is>
       </c>
     </row>
@@ -7073,7 +7077,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -7336,6 +7340,43 @@
         </is>
       </c>
       <c r="G8" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>D2</t>
+        </is>
+      </c>
+      <c r="B9" s="14" t="inlineStr">
+        <is>
+          <t>CORRECTION to the record: "clean-checkout verify is red" was attributed solely to the uncommitted model-catalog/GGUF test fixes (Decision Q6). That was incomplete. There were TWO independent causes.</t>
+        </is>
+      </c>
+      <c r="C9" s="14" t="inlineStr">
+        <is>
+          <t>Nothing now. Both causes are fixed and a clean clone verifies green.</t>
+        </is>
+      </c>
+      <c r="D9" s="14" t="inlineStr">
+        <is>
+          <t>Cause 1: the uncommitted test fixes (timezone-dependent formatDate assertions, GGUF catalog filtering) - committed 2026-09-09 as 784adb09a / 0d3c2b470 / 9621b112c after user authorisation. Cause 2, previously unrecorded and independent of Q6: every icon except src-tauri/icons/icon.png is gitignored and generated, and tauri-build needs icons/icon.ico to compile the Tauri test target, so a fresh clone died before running a single test. test-rust's TAURI_CONFIG override does NOT avoid this on Windows - measured. Fixed by f8772ec2d (generate icons when missing) and c54856d2e (stop that generation overwriting the 1024x1024 master with its own 512x512 output - the cause of the long-unexplained icon.png diff).</t>
+        </is>
+      </c>
+      <c r="E9" s="15" t="inlineStr">
+        <is>
+          <t>PROVEN, not inferred: a fresh clone of the branch, installed and built from scratch, ran make verify to exit 0 on 2026-09-09. Cause 1 alone was necessary but NOT sufficient; committing those files would not have made a clean clone green on its own.</t>
+        </is>
+      </c>
+      <c r="F9" s="13" t="inlineStr">
+        <is>
+          <t>Noted</t>
+        </is>
+      </c>
+      <c r="G9" s="13" t="inlineStr">
         <is>
           <t>2026-09-09</t>
         </is>
@@ -7426,11 +7467,19 @@
       </c>
       <c r="E2" s="13" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="F2" s="15" t="n"/>
-      <c r="G2" s="15" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F2" s="15" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="G2" s="15" t="inlineStr">
+        <is>
+          <t>contract: web-app/src/services/media/contract/{tasks,params,models,jobs,index,upcast}.ts + __tests__/{params,upcast}.test.ts, parity.test.tsx, fixtures/worker-v1-capabilities.json. v1 residue: services/atomicMedia/client{,.test}.ts. catalog: lib/models.ts, hooks/useModelSources.ts, services/models/default.ts (+3 test files). build: Makefile (app-icons). guard: scripts/selective-v2032-protected.json. docs: this tracker. No UI file changed.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="n">
@@ -7453,11 +7502,19 @@
       </c>
       <c r="E3" s="13" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="F3" s="15" t="n"/>
-      <c r="G3" s="15" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F3" s="15" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="G3" s="15" t="inlineStr">
+        <is>
+          <t>make verify exit 0 on the working tree AND on a from-scratch clean clone (2026-09-09). Web coverage 2319 passed/16 skipped; extensions 250+276; Rust 487+12+167+205+28+4; coverage floor 9 critical files; selective-v2032 boundaries verified. Nothing was skipped or unavailable in either run.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="n">
@@ -7480,11 +7537,19 @@
       </c>
       <c r="E4" s="13" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="F4" s="15" t="n"/>
-      <c r="G4" s="15" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F4" s="15" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="G4" s="15" t="inlineStr">
+        <is>
+          <t>parity.test.tsx - 6 tests, all passing. It renders the live MediaGenerationForm and asserts JSON.stringify equality of the submitted body across defaults, negative prompt + seed, a non-default resolution, the quantiser tie, and image_to_video with a reference image. Mutation-checked: flipping the tie-break from &lt;= to &lt; fails exactly one case, so the green is earned not vacuous.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="n">
@@ -7530,11 +7595,19 @@
       </c>
       <c r="E6" s="13" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="F6" s="15" t="n"/>
-      <c r="G6" s="15" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F6" s="15" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="G6" s="15" t="inlineStr">
+        <is>
+          <t>make test-selective-v2032 green. Re-baseline commits: Task 0 = 9e8249046 era (8 media files); Task 2 = 59ee8b7fb (exactly 2 entries - atomicMedia/client.ts and client.test.ts). Each re-baseline is an isolated commit containing only the manifest, per Q1.</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="26.4" customHeight="1">
       <c r="A7" s="6" t="n">
@@ -7553,11 +7626,19 @@
       </c>
       <c r="E7" s="13" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="F7" s="15" t="n"/>
-      <c r="G7" s="15" t="n"/>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F7" s="15" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="G7" s="15" t="inlineStr">
+        <is>
+          <t>PREMISE VOID as of 2026-09-09: the user authorised committing the pre-existing dirty paths, so they are no longer dirty. 8 of 11 were committed after review (784adb09a, 0d3c2b470, 9621b112c) and downloads/index.html was deleted on request (6ed0979bb). Two were reviewed and DISCARDED as damage/churn: src-tauri/icons/icon.png (a 512x512 overwrite of the 1024x1024 master - see D2) and extensions/yarn.lock (rebuild fingerprint of the locally built core tarball, re-churns on every build).</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="n">

</xml_diff>

<commit_message>
docs(tracker): record Task 4 commit and backfill missing SHAs
Marks T04-S07 done, backfills the commit SHAs for Tasks 0, 3 and 4 that were
left blank, updates the make-verify evidence with the latest numbers and the one
lint failure, and downgrades the conformance-suite evidence row to Partial: one
adapter passes it, and the phase gate asks for two.

Points the handover at T05-S01, including the instruction that the ComfyUI
adapter must pass the conformance suite unmodified.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/superpowers/plans/2026-09-08-model-agnostic-atomic-media-platform-tracker.xlsx
+++ b/docs/superpowers/plans/2026-09-08-model-agnostic-atomic-media-platform-tracker.xlsx
@@ -1081,7 +1081,7 @@
       </c>
       <c r="B7" s="22" t="inlineStr">
         <is>
-          <t>c54856d2e fix(verify): stop icon generation from degrading the icon.png master</t>
+          <t>f224ce822 feat(media): support multiple media providers (pushed)</t>
         </is>
       </c>
     </row>
@@ -1093,7 +1093,7 @@
       </c>
       <c r="B8" s="22" t="inlineStr">
         <is>
-          <t>Tasks 0-3 all Done and committed. Next work is Task 4 (T04-S01): failing store tests for the multi-provider registry - baseline present, enable/disable persists, two providers merge without id collision, disabling clears a stale selection. Note Task 4 persists to the EXISTING settings surface: no new config file, and any secret goes where cloud LLM keys go, never localStorage.</t>
+          <t>Tasks 0-4 all Done, committed and pushed. Next work is Task 5 (T05-S01): READ the ComfyUI HTTP/WS surface before writing anything (/object_info, /prompt, /history/{id}, /queue, /interrupt, /view, /ws) and record which ComfyUI version was validated against. Then build from RECORDED FIXTURES, never a live server.</t>
         </is>
       </c>
     </row>
@@ -1105,7 +1105,7 @@
       </c>
       <c r="B9" s="22" t="inlineStr">
         <is>
-          <t>Q1 Answered. Tasks 0, 1, 2, 3 Done. D1 and D2 recorded. Q2-Q6 still Open. Next not-done step: T04-S01. The adapter conformance suite at services/media/adapters/__tests__/conformance.ts is now the contract for every future provider - do not weaken it to make an adapter pass.</t>
+          <t>Q1 Answered. Tasks 0, 1, 2, 3, 4 Done. D1/D2 Noted, D3 OPEN (secrets - a security decision for the user at Task 6). Q2-Q6 still Open. Next not-done step: T05-S01.</t>
         </is>
       </c>
     </row>
@@ -1189,7 +1189,7 @@
       </c>
       <c r="B16" s="23" t="inlineStr">
         <is>
-          <t>Start Task 4 at T04-S01. Two guard re-baselines have happened so far (Task 2 and Task 3), each isolated per Q1; expect to need authorisation again if a protected file must change. Task 5 (ComfyUI) is the first real test of the abstraction, since an adapter-specific branch in the conformance suite would mean the contract is wrong.</t>
+          <t>Start Task 5 at T05-S01. It is the real test of the abstraction: the ComfyUI adapter must pass services/media/adapters/__tests__/conformance.ts UNMODIFIED. If a test needs bending to fit, the contract is underspecified and the CONTRACT changes - never the suite. Local pre-flight before any full gate: yarn lint AND tsc -b AND the focused tests (a run was lost to skipping lint). Three guard re-baselines have happened (Tasks 0, 2, 3), each isolated per Q1; authorisation is needed again for any further protected-file change.</t>
         </is>
       </c>
     </row>
@@ -1417,7 +1417,11 @@
           <t>make verify green</t>
         </is>
       </c>
-      <c r="I3" s="13" t="n"/>
+      <c r="I3" s="13" t="inlineStr">
+        <is>
+          <t>9e8249046 (in merge 8ec82bef3)</t>
+        </is>
+      </c>
       <c r="J3" s="14" t="inlineStr">
         <is>
           <t>HARD GATE. Guard is red now: 8 of 11 protected media files changed by a13b71a83. Adds scripts/rebaseline-selective-v2032.mjs.</t>
@@ -1572,7 +1576,11 @@
           <t>Two adapters pass one conformance suite</t>
         </is>
       </c>
-      <c r="I6" s="13" t="n"/>
+      <c r="I6" s="13" t="inlineStr">
+        <is>
+          <t>eda596d8d (+ abcc50d48 guard re-baseline)</t>
+        </is>
+      </c>
       <c r="J6" s="14" t="inlineStr">
         <is>
           <t>Mock transport. Writes the shared conformance suite that every later adapter must pass.</t>
@@ -1621,7 +1629,11 @@
           <t>Two adapters pass one conformance suite</t>
         </is>
       </c>
-      <c r="I7" s="13" t="n"/>
+      <c r="I7" s="13" t="inlineStr">
+        <is>
+          <t>f224ce822</t>
+        </is>
+      </c>
       <c r="J7" s="14" t="inlineStr">
         <is>
           <t>Bundled baseline is the existing local worker, so current users see no change.</t>
@@ -3646,7 +3658,7 @@
       </c>
       <c r="E35" s="13" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F35" s="13" t="n"/>
@@ -3660,7 +3672,11 @@
           <t>Laptop</t>
         </is>
       </c>
-      <c r="I35" s="15" t="n"/>
+      <c r="I35" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-09: committed f224ce822 "feat(media): support multiple media providers" and pushed. No protected file changed, so no guard re-baseline was needed this time. Full make verify exit 0.</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="26.4" customHeight="1">
       <c r="A36" s="6" t="inlineStr">
@@ -7601,7 +7617,7 @@
       </c>
       <c r="G3" s="15" t="inlineStr">
         <is>
-          <t>make verify exit 0 on the working tree AND on a from-scratch clean clone (2026-09-09). Web coverage 2319 passed/16 skipped; extensions 250+276; Rust 487+12+167+205+28+4; coverage floor 9 critical files; selective-v2032 boundaries verified. Nothing was skipped or unavailable in either run.</t>
+          <t>make verify exit 0 on the working tree at every task boundary, AND on a from-scratch clean clone (2026-09-09). Latest run: web coverage 2368 passed / 16 skipped (up from 2234 at session start); extensions 250 + 276; Rust 487 + 12 + 167 + 205 + 28 + 4; coverage floor 9 critical files; selective-v2032 boundaries verified. Nothing skipped or unavailable. One run FAILED on lint (exit 2) from an omit-by-destructuring pattern leaving unused bindings; fixed and re-run green.</t>
         </is>
       </c>
     </row>
@@ -7657,11 +7673,19 @@
       </c>
       <c r="E5" s="13" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="F5" s="15" t="n"/>
-      <c r="G5" s="15" t="n"/>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="F5" s="15" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="G5" s="15" t="inlineStr">
+        <is>
+          <t>30/30 for the Atomic Media Worker adapter. ONE adapter only - the phase gate is "two adapters pass one conformance suite", so this is half met until Task 5's ComfyUI adapter passes the same suite UNMODIFIED. An adapter-specific branch in the suite would mean the contract is wrong.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="n">

</xml_diff>

<commit_message>
docs(tracker): record the Task 5 commit SHA
Backfills 051aa223e into the Task 5 Commit SHA column and updates the
Handover sheet's "Latest local commit" row, the same way 746c75579 did
for Task 4. The SHA cannot be written in the commit it names, so it lands
here.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/superpowers/plans/2026-09-08-model-agnostic-atomic-media-platform-tracker.xlsx
+++ b/docs/superpowers/plans/2026-09-08-model-agnostic-atomic-media-platform-tracker.xlsx
@@ -1081,7 +1081,7 @@
       </c>
       <c r="B7" s="22" t="inlineStr">
         <is>
-          <t>746c75579 docs(tracker): record Task 4 commit and backfill missing SHAs (pushed). Task 5's work is in the working tree, UNCOMMITTED, awaiting the user's authorisation.</t>
+          <t>051aa223e feat(media): add ComfyUI provider adapter - COMMITTED 2026-09-09, NOT PUSHED. Branch is ahead of origin/feature/atomic-code-foundation by 1. Ask the user before pushing.</t>
         </is>
       </c>
     </row>
@@ -1193,7 +1193,6 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
     <row r="18">
       <c r="A18" s="20" t="inlineStr">
         <is>
@@ -1683,7 +1682,11 @@
           <t>Two adapters pass one conformance suite</t>
         </is>
       </c>
-      <c r="I8" s="13" t="n"/>
+      <c r="I8" s="13" t="inlineStr">
+        <is>
+          <t>051aa223e</t>
+        </is>
+      </c>
       <c r="J8" s="14" t="inlineStr">
         <is>
           <t>Fixtures only, never live. ComfyUI runs CPU-only and /object_info responds without generating.</t>

</xml_diff>

<commit_message>
docs(tracker): record the Task 7 commit SHA
Backfills 94d164c02 into the Task 7 Commit SHA column and marks the
Handover sheet's "Latest local commit" row as pushed. Same pattern as
746c75579 and ab7a28911: a commit cannot name its own SHA.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/superpowers/plans/2026-09-08-model-agnostic-atomic-media-platform-tracker.xlsx
+++ b/docs/superpowers/plans/2026-09-08-model-agnostic-atomic-media-platform-tracker.xlsx
@@ -1081,7 +1081,7 @@
       </c>
       <c r="B7" s="22" t="inlineStr">
         <is>
-          <t>051aa223e feat(media): add ComfyUI provider adapter - COMMITTED 2026-09-09, NOT PUSHED. Branch is ahead of origin/feature/atomic-code-foundation by 1. Ask the user before pushing.</t>
+          <t>94d164c02 feat(media): add cross-provider media job manager - COMMITTED AND PUSHED 2026-09-09. Branch is in sync with origin/feature/atomic-code-foundation.</t>
         </is>
       </c>
     </row>
@@ -1193,7 +1193,6 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
     <row r="18">
       <c r="A18" s="20" t="inlineStr">
         <is>
@@ -1785,7 +1784,11 @@
           <t>Job manager and library unit tests green</t>
         </is>
       </c>
-      <c r="I10" s="13" t="n"/>
+      <c r="I10" s="13" t="inlineStr">
+        <is>
+          <t>94d164c02</t>
+        </is>
+      </c>
       <c r="J10" s="14" t="inlineStr">
         <is>
           <t>Fake timers. Fixes C10, C11, C12.</t>

</xml_diff>

<commit_message>
docs(tracker): answer D3 and Q5, unblocking Task 6
D3 answered: cloud media API keys go in the OS credential store, not
localStorage. That resolves the plan's Task 4 Step 4 contradiction in
favour of "never in localStorage" and against "the same way cloud LLM
keys already are" - the latter being localStorage today.

Q5 answered, and deliberately recorded as SCOPED rather than blanket:
an ok for four named crates (keyring 4.2 plus the Windows, Apple and
Linux Secret Service backends) for credential storage only. Task 9 and
Task 8 Step 5 must still ask for their own, naming crate and reason, per
AGENTS.md rule 6.

Also recorded against Task 6 as must-settle-before-code: what keyring
does on Linux when no Secret Service daemon is running. Undocumented in
docs.rs as fetched today, and common on minimal installs.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/superpowers/plans/2026-09-08-model-agnostic-atomic-media-platform-tracker.xlsx
+++ b/docs/superpowers/plans/2026-09-08-model-agnostic-atomic-media-platform-tracker.xlsx
@@ -1105,7 +1105,7 @@
       </c>
       <c r="B9" s="22" t="inlineStr">
         <is>
-          <t>Q1 Answered. Q2 ANSWERED 2026-09-09: cloud providers ARE in scope, so Task 6 is live (deferred by the user's choice, not skipped). Tasks 0-4 Done. Task 5 In progress (only the commit step remains). D1/D2/D4 Noted. D5 Answered 2026-09-09 (Task 7 leaves useAtomicMediaJob alone - no protected file, no re-baseline). D3 is now a LIVE blocker for Task 6. Q3-Q6 still Open. Next not-done step: T05-S06, then Task 7 (T07-S01).</t>
+          <t>Q1, Q2, D3, D5, Q5 all Answered. Tasks 0-5 and 7 Done and pushed. D1/D2/D4/D6 Noted. Q3, Q4, Q6 still Open. Task 6 is now FULLY UNBLOCKED (cloud in scope; OS credential store; four keyring crates approved for credential storage only). Task 8 and Task 10 are also unblocked. Nothing is waiting on the user.</t>
         </is>
       </c>
     </row>
@@ -1189,7 +1189,7 @@
       </c>
       <c r="B16" s="23" t="inlineStr">
         <is>
-          <t>Raise D3 with the user if Task 6 is wanted next; otherwise start Task 8 (asset materialisation and the media library), which Task 7 has just unblocked. Task 10 (schema-driven parameter renderer) is also unblocked and is the plan's 'biggest single win' - it is what would make the ComfyUI adapter visible on screen.</t>
+          <t>Ask the user which he wants next - nothing is blocked now. Task 6 (cloud adapter, now fully unblocked), Task 8 (asset materialisation and the media library, unblocked by Task 7), or Task 10 (schema-driven parameter renderer - the plan calls it the biggest single win, and it is what would finally make the ComfyUI adapter visible on screen; everything built so far is invisible plumbing). If Task 6: settle the Linux no-daemon fallback FIRST.</t>
         </is>
       </c>
     </row>
@@ -1727,7 +1727,7 @@
       <c r="F9" s="13" t="n"/>
       <c r="G9" s="14" t="inlineStr">
         <is>
-          <t>Q2 (answered - cloud IS in scope); D3 must be answered before starting</t>
+          <t>Q2, D3, Q5 all answered - UNBLOCKED</t>
         </is>
       </c>
       <c r="H9" s="14" t="inlineStr">
@@ -1743,7 +1743,7 @@
       </c>
       <c r="K9" s="15" t="inlineStr">
         <is>
-          <t>2026-09-09: UNBLOCKED - Q2 answered 'yes, include cloud providers'. Deliberately DEFERRED, not skipped: the user chose Task 7 as the next piece of work. Strict tracker order would have taken Task 6 next; this deviation is the user's call, recorded here rather than made silently. Task 6 is self-contained and nothing downstream depends on it, so it can be slotted in at any point. Do NOT start it until D3 (where the API key is stored) is answered.</t>
+          <t>2026-09-09: FULLY UNBLOCKED. Q2 answered (cloud IS in scope), D3 answered (OS credential store), Q5 answered (the four keyring crates approved, for credential storage only). Not started. Before writing code: settle what keyring does on Linux with no Secret Service daemon and design the fallback. Note the user was told, and accepted, that cloud LLM api_keys remain in plaintext localStorage - hardening those is a separate piece of work he has not commissioned.</t>
         </is>
       </c>
     </row>
@@ -1888,7 +1888,11 @@
           <t>GATED on Q3. Rust spawn/stop/restart testable against a stub process.</t>
         </is>
       </c>
-      <c r="K12" s="15" t="n"/>
+      <c r="K12" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-09: still gated on Q3 (unanswered). Q5 was answered on 2026-09-09 but SCOPED to four credential-storage crates only - it is NOT approval for any dependency this task might want. Ask again, naming the crate and reason.</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="26.4" customHeight="1">
       <c r="A13" s="6" t="inlineStr">
@@ -7423,13 +7427,21 @@
           <t>Plan aims for zero. AGENTS.md 6.6 requires a name-and-reason approval; ask at the point of need rather than assuming here.</t>
         </is>
       </c>
-      <c r="E6" s="15" t="n"/>
+      <c r="E6" s="15" t="inlineStr">
+        <is>
+          <t>ANSWERED BY THE USER 2026-09-09, SCOPED - this is an ok for FOUR NAMED CRATES FOR CREDENTIAL STORAGE ONLY, not a blanket yes to new dependencies. He was shown the names, the count and the reason before answering, per AGENTS.md rule 6. Approved: keyring 4.2 (core), windows-native-keyring-store, apple-native-keyring-store, and a Linux Secret Service backend (dbus-secret-service-keyring-store or zbus-). Target-gated, so exactly one backend compiles into any given build, but four Cargo.toml entries against a plan that aimed for zero. REASON: it is what D3's answer (OS credential store) requires; keyring 4.x keeps its platform backends as separate optional crates rather than bundling them as 3.x did. STILL NEEDS ITS OWN OK: any dependency for Task 9 (worker supervision) or Task 8 Step 5. This answer does not cover them - approval for one action is never approval for the next. UNRESOLVED, MUST BE SETTLED BEFORE T06 CODE IS WRITTEN: what keyring does on Linux when no Secret Service daemon is running. Not documented in docs.rs as fetched 2026-09-09, and it is a common case on minimal installs. A fallback path is needed or those users hit an error they cannot fix. Find out for certain; do not assume.</t>
+        </is>
+      </c>
       <c r="F6" s="13" t="inlineStr">
         <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="G6" s="13" t="n"/>
+          <t>Answered</t>
+        </is>
+      </c>
+      <c r="G6" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="26.4" customHeight="1">
       <c r="A7" s="6" t="inlineStr">
@@ -7557,15 +7569,19 @@
       </c>
       <c r="E10" s="15" t="inlineStr">
         <is>
-          <t>Deferred to Task 6. Not guessed. | 2026-09-09 UPDATE: Q2 was answered 'cloud in scope', so this is now a LIVE blocker for Task 6, not a deferred hypothetical. It must be answered before T06-S02 is written.</t>
+          <t>ANSWERED BY THE USER 2026-09-09: the OS credential store (Windows Credential Manager, macOS Keychain, Linux Secret Service). NOT localStorage, which resolves the plan's contradiction in favour of the 'never in localStorage' clause and against 'the same way cloud LLM keys already are'. He was shown, and chose against, three alternatives: tauri-plugin-store (already a dependency, but plaintext on disk), localStorage (consistent with today but plaintext and readable from the web view), and never storing the key at all. Rationale given to him: it is the only option where the key is actually encrypted at rest rather than merely tucked away. CONSEQUENCE, RAISED SEPARATELY: this requires at least one new Rust runtime dependency, which AGENTS.md rule 6 says needs his explicit ok naming the crate and reason, and which is what Q5 asks. D3 is NOT blanket approval for Q5. COST OF CHANGING LATER: low for the code - the contract stores only auth.setting_key, a name, never a value, so the storage sits behind one indirection - but any keys already saved would need migrating. PRE-EXISTING AND UNTOUCHED: cloud LLM provider api_keys are in plaintext localStorage today via hooks/useModelProvider.ts, which persists its whole state with no partialize. Out of scope, but he has been told.</t>
         </is>
       </c>
       <c r="F10" s="13" t="inlineStr">
         <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="G10" s="13" t="n"/>
+          <t>Answered</t>
+        </is>
+      </c>
+      <c r="G10" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">

</xml_diff>

<commit_message>
docs(tracker): record the Task 6 commit SHA
Backfills bfc35573f, same pattern as 746c75579, ab7a28911 and 7a2753492.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/superpowers/plans/2026-09-08-model-agnostic-atomic-media-platform-tracker.xlsx
+++ b/docs/superpowers/plans/2026-09-08-model-agnostic-atomic-media-platform-tracker.xlsx
@@ -1081,7 +1081,7 @@
       </c>
       <c r="B7" s="22" t="inlineStr">
         <is>
-          <t>94d164c02 feat(media): add cross-provider media job manager - COMMITTED AND PUSHED 2026-09-09. Branch is in sync with origin/feature/atomic-code-foundation.</t>
+          <t>bfc35573f feat(media): add remote HTTP media provider adapter - COMMITTED AND PUSHED 2026-09-09.</t>
         </is>
       </c>
     </row>
@@ -1193,7 +1193,6 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
     <row r="18">
       <c r="A18" s="20" t="inlineStr">
         <is>
@@ -1736,7 +1735,11 @@
           <t>Two adapters pass one conformance suite</t>
         </is>
       </c>
-      <c r="I9" s="13" t="n"/>
+      <c r="I9" s="13" t="inlineStr">
+        <is>
+          <t>bfc35573f</t>
+        </is>
+      </c>
       <c r="J9" s="14" t="inlineStr">
         <is>
           <t>GATED on Q2. Skip entirely if local-only. Cloud does the compute, so this is ideal laptop work.</t>

</xml_diff>

<commit_message>
docs(tracker): record the Task 8 commit SHA
Backfills a635958f5.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/superpowers/plans/2026-09-08-model-agnostic-atomic-media-platform-tracker.xlsx
+++ b/docs/superpowers/plans/2026-09-08-model-agnostic-atomic-media-platform-tracker.xlsx
@@ -1081,7 +1081,7 @@
       </c>
       <c r="B7" s="22" t="inlineStr">
         <is>
-          <t>bfc35573f feat(media): add remote HTTP media provider adapter - COMMITTED AND PUSHED 2026-09-09.</t>
+          <t>a635958f5 feat(media): materialise outputs and persist a media library - COMMITTED AND PUSHED 2026-09-09.</t>
         </is>
       </c>
     </row>
@@ -1841,7 +1841,11 @@
           <t>Job manager and library unit tests green</t>
         </is>
       </c>
-      <c r="I11" s="13" t="n"/>
+      <c r="I11" s="13" t="inlineStr">
+        <is>
+          <t>a635958f5</t>
+        </is>
+      </c>
       <c r="J11" s="14" t="inlineStr">
         <is>
           <t>Mocked fs. Thumbnails are WebView2, not GPU.</t>

</xml_diff>

<commit_message>
docs(tracker): record the Task 10 commit SHA
Backfills 642223616.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/superpowers/plans/2026-09-08-model-agnostic-atomic-media-platform-tracker.xlsx
+++ b/docs/superpowers/plans/2026-09-08-model-agnostic-atomic-media-platform-tracker.xlsx
@@ -1081,7 +1081,7 @@
       </c>
       <c r="B7" s="22" t="inlineStr">
         <is>
-          <t>a635958f5 feat(media): materialise outputs and persist a media library - COMMITTED AND PUSHED 2026-09-09.</t>
+          <t>642223616 feat(media): render generation parameters from schema - COMMITTED AND PUSHED 2026-09-10.</t>
         </is>
       </c>
     </row>
@@ -1943,7 +1943,11 @@
           <t>make verify-fast green; visual parity</t>
         </is>
       </c>
-      <c r="I13" s="13" t="n"/>
+      <c r="I13" s="13" t="inlineStr">
+        <is>
+          <t>642223616</t>
+        </is>
+      </c>
       <c r="J13" s="14" t="inlineStr">
         <is>
           <t>Pure React + RTL. Biggest single win, needs nothing but a laptop.</t>

</xml_diff>

<commit_message>
docs(tracker): record Task 11 complete and its two commit SHAs
Also records D11: the re-baseline script cannot express the deletion of a
protected file, which Task 11 hit and worked around by hand.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/superpowers/plans/2026-09-08-model-agnostic-atomic-media-platform-tracker.xlsx
+++ b/docs/superpowers/plans/2026-09-08-model-agnostic-atomic-media-platform-tracker.xlsx
@@ -1081,7 +1081,7 @@
       </c>
       <c r="B7" s="22" t="inlineStr">
         <is>
-          <t>642223616 feat(media): render generation parameters from schema - COMMITTED AND PUSHED 2026-09-10.</t>
+          <t>e5ee6f793 chore(guard): re-baseline the selective v2.0.32 protected surface - 2026-09-10.</t>
         </is>
       </c>
     </row>
@@ -1093,7 +1093,7 @@
       </c>
       <c r="B8" s="22" t="inlineStr">
         <is>
-          <t>Tasks 0-8 and 10 Done. Next is Task 11 (refit the Media Studio onto the platform) - it is the first task that EDITS THE PROTECTED FILES (MediaGenerationForm.tsx, MediaStudio.tsx, useAtomicMediaJob.ts), so it needs a guard re-baseline and the user's explicit authorisation for it under the Q1 rule. It is also the task that finally makes all of this visible on screen: everything built so far is working, tested plumbing that the user cannot yet see.</t>
+          <t>Tasks 0-8, 10 and 11 Done. Task 11 is finished and the Media Studio now runs entirely on the platform - this is the first time any of Tasks 1-10 is visible on screen. Next is Task 12 (provider and model management UI, gated only on Task 4, which is Done) or Task 13 (media library route, gated on Task 8, Done). Task 9 is still gated on Q3, which is OPEN. Before Task 13, settle D8 - the unresolved-seed gap - because re-run depends on it.</t>
         </is>
       </c>
     </row>
@@ -1129,7 +1129,7 @@
       </c>
       <c r="B11" s="22" t="inlineStr">
         <is>
-          <t>2026-09-09 for Task 7: make verify EXITCODE=0 in a VS x64 developer shell. PRE-FLIGHT MUST INCLUDE 'node scripts/check-test-quality.mjs' - lint, tsc and vitest all passed while that guard was red. Environment reminder: vcvars64.bat, GnuWin32 make on PATH, plus a printf-ONLY directory that also contains msys-2.0.dll / msys-intl-8.dll / msys-iconv-2.dll (printf.exe without its msys runtime cannot start and fails one Rust shell-contract test). Do NOT add Git's usr/bin wholesale. ALWAYS read the log's own EXITCODE line - a wrapper's exit code reported 0 on three runs that were actually red.</t>
+          <t>2026-09-10 for Task 11: make verify-fast EXITCODE=0 and make test-selective-v2032 EXITCODE=0, both read from the command's own exit code. Full web suite 2442 passed / 214 files from the REPO ROOT. WARNING: run vitest from the repo root, not from web-app - src/services/__tests__/external-contracts.test.ts computes its repo root with endsWith('/web-app'), which is false on Windows backslash paths, so 9 tests fail with ENOENT for no real reason. FULL make verify was NOT run on 2026-09-10: MSVC was not on the shell's PATH and Git's link.exe shadowed it. Task 11 touches no Rust, but the full gate is still owed.</t>
         </is>
       </c>
     </row>
@@ -1189,10 +1189,11 @@
       </c>
       <c r="B16" s="23" t="inlineStr">
         <is>
-          <t>Ask the user which of those three he wants. If the credential store: settle FIRST what keyring does on Linux with no Secret Service daemon - the crate's own docs acknowledge 'known issues' in headless environments and document no automatic fallback, so a fallback must be designed rather than discovered by a user. Do NOT silently downgrade to plaintext; surface the choice.</t>
-        </is>
-      </c>
-    </row>
+          <t>Run the full make verify in a VS x64 developer shell to close out Task 11 properly - it is the one gate this session could not run. Then ask the user which of Task 12 or Task 13 he wants next, and raise Q3 if Task 9 is being considered.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17"/>
     <row r="18">
       <c r="A18" s="20" t="inlineStr">
         <is>
@@ -1982,7 +1983,7 @@
       </c>
       <c r="E14" s="13" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F14" s="13" t="n"/>
@@ -1996,7 +1997,11 @@
           <t>make verify-fast green; visual parity</t>
         </is>
       </c>
-      <c r="I14" s="13" t="n"/>
+      <c r="I14" s="13" t="inlineStr">
+        <is>
+          <t>refit + e5ee6f793 (guard re-baseline)</t>
+        </is>
+      </c>
       <c r="J14" s="14" t="inlineStr">
         <is>
           <t>EDITS THE PROTECTED FILES - Task 0 must be green first. Includes the payload-parity regression test.</t>
@@ -2004,7 +2009,7 @@
       </c>
       <c r="K14" s="15" t="inlineStr">
         <is>
-          <t>2026-09-10: S01 Done (visual-parity guard, no protected file touched). Both blockers CLEARED by the user on 2026-09-10. (1) AUTHORISED to proceed: S04-S08 edit SEVEN of the eleven protected files (MediaGenerationForm.tsx, MediaStudio.tsx, MediaPreview.tsx, MediaJobStatus.tsx, MediaStudio.test.tsx, useAtomicMediaJob.ts + its test, the last two deleted) and S10 re-baselines the guard - he gave the explicit ok for this specific task, re-baseline included, per Q1's rule. (2) Q4 ANSWERED: always materialise, CSP untouched. Verified while sizing the work, not assumed: tauri.conf.json img-src allows https: but media-src does NOT, so today's toPreviewSrc https: passthrough renders a remote IMAGE fine and silently blocks a remote VIDEO. That is the CSP bug the step note names.</t>
+          <t>2026-09-10: Task 11 COMPLETE, S01-S11 all Done. This is the task that made Tasks 1-10 visible: MODES and all eight bespoke control blocks deleted (489 lines -&gt; 293), tabs and controls now come from what providers declare, useAtomicMediaJob deleted, and Task 8's materialisation wired so generated files reach the screen. Fixes C3 (image_to_image unreachable), C5 (adding a parameter meant editing a frozen file), C10 (job died with the component) and C11 (cancel was a no-op). TWO REAL DEFECTS CAUGHT BY TESTS, NOT REVIEW: the refit initially dropped the device default, which would have silently changed every submitted body - found by the rewritten parity test; and the test-quality guard caught two of this task's own tests asserting nothing but mock invocation, which were strengthened rather than allowlisted. Payload parity is PROVEN end to end: parity.test.tsx drives the real refitted form through the real downcaster and asserts a byte-identical v1 body. Visual parity was redefined once, deliberately, under D10. Gate: make verify-fast EXITCODE=0, make test-selective-v2032 EXITCODE=0, media suite 832, full web suite 2442 (baseline 2416, so +26). FULL make verify NOT run in this session - it needs MSVC for the Rust side and the shell had Git's link.exe shadowing it; this task touches no Rust.</t>
         </is>
       </c>
     </row>
@@ -5699,7 +5704,7 @@
       </c>
       <c r="I84" s="15" t="inlineStr">
         <is>
-          <t>2026-09-10 Guard confirmed RED first, exit code 1 read from the script itself rather than a wrapper: 5 protected files changed, 2 missing (deleted). Re-baselined in its own isolated single-purpose commit, per Q1's rule.</t>
+          <t>2026-09-10 Guard confirmed RED first, exit code 1 read from the script itself rather than a wrapper: 5 protected files changed, 2 missing (deleted). Re-baselined in its own isolated single-purpose commit, per Q1's rule. BLOCKED BRIEFLY BY A TOOL GAP, recorded as D11: the re-baseline script throws 'Protected file missing' and writes nothing when a protected file has been DELETED, so the two useAtomicMediaJob entries had to be removed from the manifest by hand before it would run.</t>
         </is>
       </c>
     </row>
@@ -5724,7 +5729,7 @@
       </c>
       <c r="E85" s="13" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F85" s="13" t="n"/>
@@ -5738,7 +5743,11 @@
           <t>Laptop</t>
         </is>
       </c>
-      <c r="I85" s="15" t="n"/>
+      <c r="I85" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-10 Done, two commits as required. (1) feat(media): drive the Media Studio from the provider platform. (2) chore(guard): re-baseline the selective v2.0.32 protected surface - isolated and single-purpose per Q1, naming the five files re-hashed and the two removed. After the re-baseline: make verify-fast EXITCODE=0 and make test-selective-v2032 EXITCODE=0.</t>
+        </is>
+      </c>
     </row>
     <row r="86" ht="26.4" customHeight="1">
       <c r="A86" s="6" t="inlineStr">
@@ -7369,7 +7378,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -7989,6 +7998,43 @@
         </is>
       </c>
       <c r="G17" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>D11</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>TOOL GAP, found while re-baselining for Task 11. scripts/rebaseline-selective-v2032.mjs cannot express the DELETION of a protected file: it iterates the manifest, throws 'Protected file missing' on the first entry whose file is absent, and writes nothing at all. A task that legitimately removes a protected file therefore cannot use the tool the plan tells it to use.</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Nothing now - worked around. It will block the next task that deletes a protected file, in exactly the same way.</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Task 0 wrote the script for files that CHANGE, which was the only case that had arisen; Task 11 is the first task to delete one. Worked around by removing the two useAtomicMediaJob entries from scripts/selective-v2032-protected.json by hand, then running the script to re-hash the remaining nine. Left as-is rather than fixed in passing: Q1 requires the re-baseline commit to be isolated and single-purpose, so changing the script in it would have broken that rule. The fix, if wanted, is a --drop &lt;path&gt; flag so a deletion is expressed in the tool and shows up in the diff rather than being hand-edited.</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Agent judgement, 2026-09-10. Recorded rather than hidden, and named in the re-baseline commit message so the next agent meets it before the script does.</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Noted</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
         <is>
           <t>2026-09-10</t>
         </is>

</xml_diff>

<commit_message>
docs(tracker): record the v2.0.35 sync outcome and decisions D19-D20
Task 19 is 10 of 11 steps done. S09, the inference smoke test, is marked
Blocked rather than skipped: ATO-465 reworked context fitting, KV-cache
estimation and OOM retry, and this machine has no model to smoke it with,
so it stays the one unverified behavioural risk of the sync.

D19 records the jsdom/undici AbortSignal mismatch and the fetch shim that
resolves it, including the residual risk that two upstream tests now depend
on raw.githubusercontent.com being reachable. D20 records splitting an
upstream test that could never pass on Windows.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/superpowers/plans/2026-09-08-model-agnostic-atomic-media-platform-tracker.xlsx
+++ b/docs/superpowers/plans/2026-09-08-model-agnostic-atomic-media-platform-tracker.xlsx
@@ -8003,7 +8003,7 @@
       </c>
       <c r="E137" s="13" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F137" s="13" t="inlineStr"/>
@@ -8017,6 +8017,11 @@
           <t>Laptop</t>
         </is>
       </c>
+      <c r="I137" t="inlineStr">
+        <is>
+          <t>PR #3 then PR #2 landed into main before branching.</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="6" t="inlineStr">
@@ -8039,7 +8044,7 @@
       </c>
       <c r="E138" s="13" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F138" s="13" t="inlineStr"/>
@@ -8053,6 +8058,11 @@
           <t>Laptop</t>
         </is>
       </c>
+      <c r="I138" t="inlineStr">
+        <is>
+          <t>Branched off main; upstream remote already present.</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="6" t="inlineStr">
@@ -8075,7 +8085,7 @@
       </c>
       <c r="E139" s="13" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F139" s="13" t="inlineStr"/>
@@ -8089,6 +8099,11 @@
           <t>Laptop</t>
         </is>
       </c>
+      <c r="I139" t="inlineStr">
+        <is>
+          <t>Merged upstream/main @64758ea - v2.0.35 plus the 12 commits after the tag. 751 files changed.</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="6" t="inlineStr">
@@ -8111,7 +8126,7 @@
       </c>
       <c r="E140" s="13" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F140" s="13" t="inlineStr"/>
@@ -8125,6 +8140,11 @@
           <t>Laptop</t>
         </is>
       </c>
+      <c r="I140" t="inlineStr">
+        <is>
+          <t>81 files needed a hand resolution. Judgement calls: SettingsMenu keeps Media and drops our MCP entry (upstream moved MCP to Connectors); models.ts restores mmproj into upstream new anchored regex; i18n/context.ts honours defaultValue; NavMain gains the standalone Media item.</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="6" t="inlineStr">
@@ -8147,7 +8167,7 @@
       </c>
       <c r="E141" s="13" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F141" s="13" t="inlineStr"/>
@@ -8161,6 +8181,11 @@
           <t>Laptop</t>
         </is>
       </c>
+      <c r="I141" t="inlineStr">
+        <is>
+          <t>PREREQUISITE HELD. "Selective v2.0.32 boundaries verified". Every Radium Media file is byte-identical to main; the two changed "media" paths are upstream own GAIA agent media tools, not ours.</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="6" t="inlineStr">
@@ -8183,7 +8208,7 @@
       </c>
       <c r="E142" s="13" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F142" s="13" t="inlineStr"/>
@@ -8197,6 +8222,11 @@
           <t>Laptop</t>
         </is>
       </c>
+      <c r="I142" t="inlineStr">
+        <is>
+          <t>verify-fast exit 0; clippy-rust exit 0; 823 Rust tests + plugins pass; selective guard passes; 3358 web tests pass (291 files, 0 failed).</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="6" t="inlineStr">
@@ -8219,7 +8249,7 @@
       </c>
       <c r="E143" s="13" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F143" s="13" t="inlineStr"/>
@@ -8233,6 +8263,11 @@
           <t>Laptop</t>
         </is>
       </c>
+      <c r="I143" t="inlineStr">
+        <is>
+          <t>cargo clippy --fix applied nothing (duplicate lib/lib-test suggestions block it), so the 18 findings were cleared by hand. 15 mechanical; the rest were dead-on-Windows-only code (sanitize_std_command, PTY test helpers) gated at their real cfg condition rather than deleted.</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="6" t="inlineStr">
@@ -8255,7 +8290,7 @@
       </c>
       <c r="E144" s="13" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F144" s="13" t="inlineStr"/>
@@ -8269,6 +8304,11 @@
           <t>Laptop</t>
         </is>
       </c>
+      <c r="I144" t="inlineStr">
+        <is>
+          <t>Media suites unchanged and green inside the full web run. The --ignored os_credential_store_round_trip passes against the real Windows Credential Manager after the merge.</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="6" t="inlineStr">
@@ -8291,7 +8331,7 @@
       </c>
       <c r="E145" s="13" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Blocked</t>
         </is>
       </c>
       <c r="F145" s="13" t="inlineStr"/>
@@ -8305,6 +8345,11 @@
           <t>Laptop + a model</t>
         </is>
       </c>
+      <c r="I145" t="inlineStr">
+        <is>
+          <t>NOT DONE - needs a model on disk, which this machine does not have. ATO-465 reworked context fitting, KV-cache estimation and OOM retry, so this remains the one unverified behavioural risk of the sync. Must be smoked before any release build.</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="6" t="inlineStr">
@@ -8327,7 +8372,7 @@
       </c>
       <c r="E146" s="13" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F146" s="13" t="inlineStr"/>
@@ -8341,6 +8386,11 @@
           <t>Laptop</t>
         </is>
       </c>
+      <c r="I146" t="inlineStr">
+        <is>
+          <t>No bump needed: the merge brought package/tauri.conf/web-app to 2.0.35 and Cargo to 0.6.599, matching upstream exactly.</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="6" t="inlineStr">
@@ -8363,7 +8413,7 @@
       </c>
       <c r="E147" s="13" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="F147" s="13" t="inlineStr"/>
@@ -8375,6 +8425,11 @@
       <c r="H147" s="6" t="inlineStr">
         <is>
           <t>Laptop</t>
+        </is>
+      </c>
+      <c r="I147" t="inlineStr">
+        <is>
+          <t>Merge committed as a true two-parent merge commit. PR still to open.</t>
         </is>
       </c>
     </row>
@@ -8395,7 +8450,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:G27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -9325,6 +9380,80 @@
       <c r="G25" t="inlineStr">
         <is>
           <t>2026-09-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>D19</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>TEST-ENVIRONMENT DEFECT exposed by the v2.0.35 sync, fixed in web-app/src/test/setup.ts. jsdom supplies AbortSignal, but the fetch it installs is undici's, and undici brand-checks the signal against the AbortSignal class it captured BEFORE jsdom replaced the global. The two are different class objects, so every real fetch(url, {signal}) in the app died under vitest on "Expected signal to be an instance of AbortSignal".</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Two upstream DropdownModelProvider tests. The provider registry seeds from a bundled baseline that does NOT contain openai, so it depends on its network refresh to learn that openai is a catalogue provider. With the fetch dead, the refresh fell back to baseline, openai looked like a custom provider, and the picker showed a section for a cloud provider the user had never connected.</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Translate rather than brand-check: run the fetch without the signal and race it against the signal's own abort event, so callers still see an AbortError at the right moment. Node's original classes are genuinely unreachable from inside the test realm - deleting the jsdom globals leaves undefined, and the classes reached via Request are jsdom's too. The honest cost is that the underlying request is no longer cancelled at the socket, which costs a test suite nothing.</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>DONE 2026-09-11 as part of the sync. NOTE THE RESIDUAL RISK, which is upstream's design and not introduced here: those two tests now pass only when raw.githubusercontent.com is reachable, because that is where the registry learns about openai. They will fail offline. Worth raising upstream rather than working around locally.</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Answered</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>D20</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>UPSTREAM TEST NOT PORTABLE TO WINDOWS, found by the v2.0.35 sync. process_tools_reject_unknown_ids_and_bad_signals spawns a real `sleep` through the agent PTY. Windows has no path for that spawn and no `sleep` program, so the test cannot pass here. Every sibling test in the file that spawns a process is already #[cfg(unix)]; this one was missed, probably because it is mostly error-path assertions with one spawn at the end.</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>make verify on Windows. It was the last red test after the merge.</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Split rather than gate wholesale. The unknown-id and bad-argument rejection assertions are portable and valuable, so they stay ungated and keep running on Windows; only the half that needs a process that really starts moves into a new #[cfg(unix)] test. proc_id_of is gated with it, since only spawning tests use it.</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>DONE 2026-09-11. Costs a small divergence from upstream in their test file, which is merge debt to carry; the alternative was losing Windows coverage of the rejection paths entirely. Worth offering upstream as a patch.</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Answered</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(tracker): mark T19-S11 done, PR #4 opened
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/superpowers/plans/2026-09-08-model-agnostic-atomic-media-platform-tracker.xlsx
+++ b/docs/superpowers/plans/2026-09-08-model-agnostic-atomic-media-platform-tracker.xlsx
@@ -8413,7 +8413,7 @@
       </c>
       <c r="E147" s="13" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F147" s="13" t="inlineStr"/>
@@ -8429,7 +8429,7 @@
       </c>
       <c r="I147" t="inlineStr">
         <is>
-          <t>Merge committed as a true two-parent merge commit. PR still to open.</t>
+          <t>Merge committed as a true two-parent merge commit (c81c4ea9). PR #4 opened against walladanger/Atomic-Chat main.</t>
         </is>
       </c>
     </row>

</xml_diff>